<commit_message>
chore(roster): add test accounts (student.test..05) to student import excel and csv files
</commit_message>
<xml_diff>
--- a/danh_sach_sinh_vien_import.xlsx
+++ b/danh_sach_sinh_vien_import.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>STT</t>
   </si>
@@ -23,6 +23,51 @@
   </si>
   <si>
     <t>Email FPT</t>
+  </si>
+  <si>
+    <t>SE170001</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn Nam (Trưởng nhóm)</t>
+  </si>
+  <si>
+    <t>student.test@fpt.edu.vn</t>
+  </si>
+  <si>
+    <t>SE170002</t>
+  </si>
+  <si>
+    <t>Trần Thị Minh Anh (Thành viên)</t>
+  </si>
+  <si>
+    <t>student.test02@fpt.edu.vn</t>
+  </si>
+  <si>
+    <t>SE170003</t>
+  </si>
+  <si>
+    <t>Lê Hoàng Long (Thành viên Tester)</t>
+  </si>
+  <si>
+    <t>student.test03@fpt.edu.vn</t>
+  </si>
+  <si>
+    <t>SE170004</t>
+  </si>
+  <si>
+    <t>Phạm Đức Lười (Cảnh báo Free-rider BR-05)</t>
+  </si>
+  <si>
+    <t>student.test04@fpt.edu.vn</t>
+  </si>
+  <si>
+    <t>SE170005</t>
+  </si>
+  <si>
+    <t>Hoàng Minh Đức (Thành viên 05)</t>
+  </si>
+  <si>
+    <t>student.test05@fpt.edu.vn</t>
   </si>
   <si>
     <t>SE170101</t>
@@ -129,30 +174,17 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F4F7"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -160,63 +192,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1F4E79"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF1F4E79"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF1F4E79"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF1F4E79"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD3D3D3"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD3D3D3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD3D3D3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD3D3D3"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,16 +538,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,144 +561,214 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(roster): remove parenthetical labels from student names
</commit_message>
<xml_diff>
--- a/danh_sach_sinh_vien_import.xlsx
+++ b/danh_sach_sinh_vien_import.xlsx
@@ -28,7 +28,7 @@
     <t>SE170001</t>
   </si>
   <si>
-    <t>Nguyễn Văn Nam (Trưởng nhóm)</t>
+    <t>Nguyễn Văn Nam</t>
   </si>
   <si>
     <t>student.test@fpt.edu.vn</t>
@@ -37,7 +37,7 @@
     <t>SE170002</t>
   </si>
   <si>
-    <t>Trần Thị Minh Anh (Thành viên)</t>
+    <t>Trần Thị Minh Anh</t>
   </si>
   <si>
     <t>student.test02@fpt.edu.vn</t>
@@ -46,7 +46,7 @@
     <t>SE170003</t>
   </si>
   <si>
-    <t>Lê Hoàng Long (Thành viên Tester)</t>
+    <t>Lê Hoàng Long</t>
   </si>
   <si>
     <t>student.test03@fpt.edu.vn</t>
@@ -55,7 +55,7 @@
     <t>SE170004</t>
   </si>
   <si>
-    <t>Phạm Đức Lười (Cảnh báo Free-rider BR-05)</t>
+    <t>Phạm Đức Nam</t>
   </si>
   <si>
     <t>student.test04@fpt.edu.vn</t>
@@ -64,7 +64,7 @@
     <t>SE170005</t>
   </si>
   <si>
-    <t>Hoàng Minh Đức (Thành viên 05)</t>
+    <t>Hoàng Minh Đức</t>
   </si>
   <si>
     <t>student.test05@fpt.edu.vn</t>

</xml_diff>